<commit_message>
chore: update FIFA World Cup 2026 data
</commit_message>
<xml_diff>
--- a/fifa/fifa_data.xlsx
+++ b/fifa/fifa_data.xlsx
@@ -721,27 +721,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Two FIFA officials get lifetime bans for misuse of funds</t>
+          <t>Messi tracker: Goals, assists, key moments in 2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>FIFA judges imposed life bans on two former federation presidents for financial misconduct.</t>
+          <t>ESPN provides game-by-game analysis of Lionel Messi's performances for Inter Miami and Argentina.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://a.espncdn.com/photo/2026/0701/r1682659_1296x729_16-9.jpg</t>
+          <t>https://a.espncdn.com/photo/2026/0617/r1674593_1296x729_16-9.jpg</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.espn.com/soccer/story/_/id/49905396/two-fifa-officials-get-life-bans-misuse-funds</t>
+          <t>https://www.espn.com/soccer/story/_/id/47978642/lionel-messi-2026-tracker-inter-miami-argentina-games-goals-assists-stats</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -753,27 +753,27 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>FIFA: 2030 World Cup final host country decision to be made 'in due course'</t>
+          <t>Ecuador hires Marcelo Gallardo through 2030 World Cup</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>FIFA said on Thursday that the decision over whether Morocco or Spain would host the 2030 World Cup final would be made "in due course."</t>
+          <t>Marcelo Gallardo, one of the most decorated coaches in the history of the Argentine league, has reached an agreement to manage Ecuador ahead of the 2030 FIFA World Cup.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://a.espncdn.com/photo/2026/0313/r1627854_1296x729_16-9.jpg</t>
+          <t>https://a.espncdn.com/photo/2026/0914/r1716613_1024x576_16-9.jpg</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.espn.com/soccer/story/_/id/49892754/fifa-decision-morocco-vs-spain-host-2030-world-cup-final-made-due-course</t>
+          <t>https://www.espn.com/soccer/story/_/id/49941399/ecuador-hires-marcelo-gallardo-2030-world-cup</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -785,27 +785,27 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026 Ballon d'Or: Full men's, women's short lists, host city change, more</t>
+          <t>Two FIFA officials get lifetime bans for misuse of funds</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>The 2026 Ballon d'Or short lists are out. Here's who could win the biggest individual prizes in men's and women's soccer.</t>
+          <t>FIFA judges imposed life bans on two former federation presidents for financial misconduct.</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://a.espncdn.com/photo/2026/0908/r1713144_2_1296x729_16-9.jpg</t>
+          <t>https://a.espncdn.com/photo/2026/0701/r1682659_1296x729_16-9.jpg</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.espn.com/soccer/story/_/id/49867974/2026-ballon-dor-full-mens-women-shortlists-host-city-change-vozinha-more</t>
+          <t>https://www.espn.com/soccer/story/_/id/49905396/two-fifa-officials-get-life-bans-misuse-funds</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -817,22 +817,22 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Messi tracker: Goals, assists, key moments in 2026</t>
+          <t>FIFA: 2030 World Cup final host country decision to be made 'in due course'</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ESPN provides game-by-game analysis of Lionel Messi's performances for Inter Miami and Argentina.</t>
+          <t>FIFA said on Thursday that the decision over whether Morocco or Spain would host the 2030 World Cup final would be made "in due course."</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://a.espncdn.com/photo/2026/0617/r1674593_1296x729_16-9.jpg</t>
+          <t>https://a.espncdn.com/photo/2026/0313/r1627854_1296x729_16-9.jpg</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.espn.com/soccer/story/_/id/47978642/lionel-messi-2026-tracker-inter-miami-argentina-games-goals-assists-stats</t>
+          <t>https://www.espn.com/soccer/story/_/id/49892754/fifa-decision-morocco-vs-spain-host-2030-world-cup-final-made-due-course</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -849,27 +849,27 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Burley: Kane should win the 2026 men's Ballon d'Or</t>
+          <t>2026 Ballon d'Or: Full men's, women's short lists, host city change, more</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Burley: Kane should win the 2026 men's Ballon d'Or</t>
+          <t>The 2026 Ballon d'Or short lists are out. Here's who could win the biggest individual prizes in men's and women's soccer.</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://espnmedia-cdn.akamaized.net/espn/media/common/2026/0909/dm_260909_COM_SOC_Analysis_Burley_Kane_should_win_the_2026_mens_Ballon_dOr_20260909_GLOBAL/dm_260909_COM_SOC_Analysis_Burley_Kane_should_win_the_2026_mens_Ballon_dOr_20260909_GLOBAL.jpg</t>
+          <t>https://a.espncdn.com/photo/2026/0908/r1713144_2_1296x729_16-9.jpg</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.espn.com/video/clip/_/id/49877552/kane-win-2026-men-ballon-dor</t>
+          <t>https://www.espn.com/soccer/story/_/id/49867974/2026-ballon-dor-full-mens-women-shortlists-host-city-change-vozinha-more</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -881,22 +881,22 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Popovic comfortable with Socceroos penalty shootout choices at World Cup</t>
+          <t>Burley: Kane should win the 2026 men's Ballon d'Or</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Socceroos coach Tony Popovic isn't second-guessing the shootout that saw his side eliminated from the FIFA World Cup, saying that he would have made the same choices had the two sides come back the next day.</t>
+          <t>Burley: Kane should win the 2026 men's Ballon d'Or</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://a.espncdn.com/photo/2026/0908/r1713099_1296x729_16-9.jpg</t>
+          <t>https://espnmedia-cdn.akamaized.net/espn/media/common/2026/0909/dm_260909_COM_SOC_Analysis_Burley_Kane_should_win_the_2026_mens_Ballon_dOr_20260909_GLOBAL/dm_260909_COM_SOC_Analysis_Burley_Kane_should_win_the_2026_mens_Ballon_dOr_20260909_GLOBAL.jpg</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.espn.com/soccer/story/_/id/49865329/popovic-comfortable-socceroos-penalty-shootout-choices-world-cup</t>
+          <t>https://www.espn.com/video/clip/_/id/49877552/kane-win-2026-men-ballon-dor</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -913,27 +913,27 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Cape Verde's Vozinha nominated for Goalkeeper of the Year award at Ballon d'Or after World Cup heroics</t>
+          <t>Popovic comfortable with Socceroos penalty shootout choices at World Cup</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Cape Verde goalkeeper Vozinha has been nominated for the men's Goalkeeper of the Year award at the 2026 Ballon d'Or.</t>
+          <t>Socceroos coach Tony Popovic isn't second-guessing the shootout that saw his side eliminated from the FIFA World Cup, saying that he would have made the same choices had the two sides come back the next day.</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://a.espncdn.com/photo/2026/0908/r1713164_1296x729_16-9.jpg</t>
+          <t>https://a.espncdn.com/photo/2026/0908/r1713099_1296x729_16-9.jpg</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.espn.com/soccer/story/_/id/49868020/cape-verde-colo-colo-vozinha-nominated-goalkeeper-year-award</t>
+          <t>https://www.espn.com/soccer/story/_/id/49865329/popovic-comfortable-socceroos-penalty-shootout-choices-world-cup</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -945,27 +945,27 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Belgian FA won't back Infantino's FIFA reelection, cites Balogun red card ban U-turn</t>
+          <t>Cape Verde's Vozinha nominated for Goalkeeper of the Year award at Ballon d'Or after World Cup heroics</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>The Belgian football federation said it can't support Gianni Infantino's bid for another term as FIFA president, citing transparency and governance issues and the way FIFA handled clearing Folarin Balogun from a mandatory one-game ban at the World Cup.</t>
+          <t>Cape Verde goalkeeper Vozinha has been nominated for the men's Goalkeeper of the Year award at the 2026 Ballon d'Or.</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://a.espncdn.com/photo/2026/0907/r1712695_1296x729_16-9.jpg</t>
+          <t>https://a.espncdn.com/photo/2026/0908/r1713164_1296x729_16-9.jpg</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.espn.com/soccer/story/_/id/49857842/gianni-infantino-fifa-belgian-fa-belgium-world-cup-2026-folarin-balogun-red-card-overturned-usmnt</t>
+          <t>https://www.espn.com/soccer/story/_/id/49868020/cape-verde-colo-colo-vozinha-nominated-goalkeeper-year-award</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -977,22 +977,22 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>FIFA president Gianni Infantino to stand for reelection in 2027</t>
+          <t>Belgian FA won't back Infantino's FIFA reelection, cites Balogun red card ban U-turn</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Gianni Infantino will run for reelection as FIFA president despite uncertainty over his future in the position following his failed attempt to raise $20 billion with the sale of a stake in future World Cups to private investors.</t>
+          <t>The Belgian football federation said it can't support Gianni Infantino's bid for another term as FIFA president, citing transparency and governance issues and the way FIFA handled clearing Folarin Balogun from a mandatory one-game ban at the World Cup.</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://a.espncdn.com/photo/2026/0906/r1712226_1296x729_16-9.jpg</t>
+          <t>https://a.espncdn.com/photo/2026/0907/r1712695_1296x729_16-9.jpg</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://www.espn.com/soccer/story/_/id/49847747/fifa-president-gianni-infantino-stand-re-election-2027</t>
+          <t>https://www.espn.com/soccer/story/_/id/49857842/gianni-infantino-fifa-belgian-fa-belgium-world-cup-2026-folarin-balogun-red-card-overturned-usmnt</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1009,27 +1009,27 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Maresca: Enzo Fernandez is 'a winner'</t>
+          <t>FIFA president Gianni Infantino to stand for reelection in 2027</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Maresca: Enzo Fernandez is 'a winner'</t>
+          <t>Gianni Infantino will run for reelection as FIFA president despite uncertainty over his future in the position following his failed attempt to raise $20 billion with the sale of a stake in future World Cups to private investors.</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://espnmedia-cdn.akamaized.net/espn/media/common/2026/0904/dm_260904_Maresca_Enzo_Fernandez_is_a_winner/dm_260904_Maresca_Enzo_Fernandez_is_a_winner.jpg</t>
+          <t>https://a.espncdn.com/photo/2026/0906/r1712226_1296x729_16-9.jpg</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://www.espn.com/video/clip/_/id/49824937/enzo-fernandez-winner</t>
+          <t>https://www.espn.com/soccer/story/_/id/49847747/fifa-president-gianni-infantino-stand-re-election-2027</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1041,27 +1041,27 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>FIFA accuses UEFA of 'smear campaign' in opposing discovery request</t>
+          <t>Maresca: Enzo Fernandez is 'a winner'</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>FIFA accused European soccer body UEFA of a "smear campaign" in a court filing Thursday concerning FIFA president Gianni Infantino's failed plan to sell stakes in the World Cup and other competitions.</t>
+          <t>Maresca: Enzo Fernandez is 'a winner'</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://a.espncdn.com/photo/2026/0903/r1711044_1296x729_16-9.jpg</t>
+          <t>https://espnmedia-cdn.akamaized.net/espn/media/common/2026/0904/dm_260904_Maresca_Enzo_Fernandez_is_a_winner/dm_260904_Maresca_Enzo_Fernandez_is_a_winner.jpg</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.espn.com/soccer/story/_/id/49817156/fifa-uefa-legal-filing-discovery-world-cup-sell-stake</t>
+          <t>https://www.espn.com/video/clip/_/id/49824937/enzo-fernandez-winner</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1073,27 +1073,27 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Socceroos transfer tracker: Where Australia's stars will play in 2026-27</t>
+          <t>FIFA accuses UEFA of 'smear campaign' in opposing discovery request</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Transfer deadlines are hitting across the globe and, with it, bringing to an end a window that has seen a remarkable surge in interest in players who represented the Socceroos at the FIFA World Cup.</t>
+          <t>FIFA accused European soccer body UEFA of a "smear campaign" in a court filing Thursday concerning FIFA president Gianni Infantino's failed plan to sell stakes in the World Cup and other competitions.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://a.espncdn.com/photo/2026/0902/r1710219_1295x729_16-9.png</t>
+          <t>https://a.espncdn.com/photo/2026/0903/r1711044_1296x729_16-9.jpg</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.espn.com/soccer/story/_/id/49466177/socceroos-transfer-tracker-where-australias-stars-play-2026-27</t>
+          <t>https://www.espn.com/soccer/story/_/id/49817156/fifa-uefa-legal-filing-discovery-world-cup-sell-stake</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1105,27 +1105,27 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Kushner says he regrets role in FIFA's World Cup sell-off plan</t>
+          <t>Socceroos transfer tracker: Where Australia's stars will play in 2026-27</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>FIFA's intended investment partner, Josh Kushner, said he regrets getting involved in Gianni Infantino's failed World Cup sell-off plan.</t>
+          <t>Transfer deadlines are hitting across the globe and, with it, bringing to an end a window that has seen a remarkable surge in interest in players who represented the Socceroos at the FIFA World Cup.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://a.espncdn.com/photo/2026/0901/r1710146_1296x729_16-9.jpg</t>
+          <t>https://a.espncdn.com/photo/2026/0902/r1710219_1295x729_16-9.png</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.espn.com/soccer/story/_/id/49796943/fifa-world-cup-sell-josh-kushner-gianni-infantino</t>
+          <t>https://www.espn.com/soccer/story/_/id/49466177/socceroos-transfer-tracker-where-australias-stars-play-2026-27</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1137,22 +1137,22 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Gomez: Nobody should wear the Argentina No. 10 jersey for quite some time!</t>
+          <t>Kushner says he regrets role in FIFA's World Cup sell-off plan</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Gomez: Nobody should wear the Argentina No. 10 jersey for quite some time!</t>
+          <t>FIFA's intended investment partner, Josh Kushner, said he regrets getting involved in Gianni Infantino's failed World Cup sell-off plan.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://espnmedia-cdn.akamaized.net/espn/media/common/2026/0901/dm_260901_Gomez_Nobody_should_wear_the_Argentina_number_10_jersey_for_quite_some_time/dm_260901_Gomez_Nobody_should_wear_the_Argentina_number_10_jersey_for_quite_some_time.jpg</t>
+          <t>https://a.espncdn.com/photo/2026/0901/r1710146_1296x729_16-9.jpg</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.espn.com/video/clip/_/id/49793781/wear-argentina-no-10-jersey-quite-some</t>
+          <t>https://www.espn.com/soccer/story/_/id/49796943/fifa-world-cup-sell-josh-kushner-gianni-infantino</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1169,27 +1169,27 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Lionel Messi's Argentina career: the stats, records and how he compares to Cristiano Ronaldo</t>
+          <t>Gomez: Nobody should wear the Argentina No. 10 jersey for quite some time!</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>After Lionel Messi announced his international retirement, ESPN takes a look at the numbers behind his storied Argentina career.</t>
+          <t>Gomez: Nobody should wear the Argentina No. 10 jersey for quite some time!</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://a.espncdn.com/photo/2026/0831/r1709497_1296x729_16-9.jpg</t>
+          <t>https://espnmedia-cdn.akamaized.net/espn/media/common/2026/0901/dm_260901_Gomez_Nobody_should_wear_the_Argentina_number_10_jersey_for_quite_some_time/dm_260901_Gomez_Nobody_should_wear_the_Argentina_number_10_jersey_for_quite_some_time.jpg</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.espn.com/soccer/story/_/id/49784066/lionel-messi-argentina-career-stats-records-how-compares-cristiano-ronaldo</t>
+          <t>https://www.espn.com/video/clip/_/id/49793781/wear-argentina-no-10-jersey-quite-some</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">

</xml_diff>